<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.002-04 Raphaël laisse le temps à Nina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.002-04.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.002-04.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La poule du marché</t>
+          <t>Raphaël laisse le temps à Nina</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>marché</t>
+          <t>marché : étals, toile, balance, fraises, sac en papier, poule, poires, tentes</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mila, Aniss, papa</t>
+          <t>Raphaël, Nina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Au marché, Aniss veut raconter la poule. Mila connaît le mot. Elle attend. Plus tard, Aniss choisit une poire, tout doucement.</t>
+          <t>Une goutte glisse sur la balance. Au bord, un éclat d'étal brille. Raphaël connaît le mot de la poule, maintenant. Nina s'arrête. Il ouvre la bouche, dit trop vite. Sourire parti, poitrine, papa accroupi. Il referme, attend. Merci vécu. Aux poires, sac trop vite, tente qui claque, mot qui tombe. Il revoit l'éclat. Un éclat d'étal tient au bord.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les tentes du marché claquent un peu au vent. Une caisse de fraises est rouge comme des perles. Un sac en papier froisse, crac. Au loin, une poule fait cot-cot. Ça sent la terre et le pain. On reste près de moi, Mila. Tu tiens le bord du panier ? Oui, papa. Il est rêche. En ce moment, Mila marche entre les étals. Le sol est un peu collant, entre les caisses. On s'arrête près des fraises. Elles sentent fort, tu trouves ? Oui. Elles sont toutes rouges. Aniss marche à côté, le sac à la main. Une plume jaune a glissé sous une caisse. J'ai vu... Aniss s'arrête. Il cherche le mot. Mila a entendu la poule, elle aussi. Elle ouvre la bouche. On peut laisser le temps, Mila. On attend la fin de la phrase. Mila referme la bouche. Elle tient le panier plus fort. Elle compte dans sa tête. Un. Deux. Trois. Le sac d'Aniss froisse encore. J'ai vu une poule. Elle faisait cot-cot. Oui. Cot-cot. Bravo, Mila. Tu as su attendre. Ils avancent vers les poires. Les poires sont vertes, un peu bosselées. Je veux... Aniss cherche encore. Mila attend encore. Une tente claque au-dessus d'eux. Je veux une poire. Une poire, d'accord. Mila, tu as écouté jusqu'au bout ? Oui, papa. On laisse le temps. Papa prend une poire dans le papier. Le papier est un peu rêche aussi. Elle est... Mila attend la fin. Elle est douce. Douce, oui. Vous parlez l'un après l'autre. On a fini près de cet étal ? Oui. On peut rentrer. Le panier est un peu lourd, maintenant. Les fraises sentent fort, tout près. On compte les poires, Mila ? Une. Deux. Et... Mila attend. Et trois. Tu as encore attendu la fin.</t>
+          <t>Une goutte glisse sur le métal de la balance. Elle brille, papa. Tu la vois, Raphaël ? Oui, papa. La goutte s'étire, puis tombe sur la toile. Elle a fait un rond. La toile est tendue, Raphaël ? Oui, maman. Ça sent le pain chaud, tout près. Ça sent le pain, papa. Tu le sens, toi ? Oui, fort. Des fraises rouges tiennent sur la toile. Elles sont lisses. Elles sentent fort, tu trouves ? Oui, maman. Au bord, un éclat d'étal brille. Il brille, papa. Tu le vois, ce petit point ? Oui, un petit point. Un sac en papier froisse, crac. Il est rêche. Tu le tiens, Raphaël ? Oui, maman. Au loin, une poule fait cot-cot. J'entends la poule ! Elle est derrière l'étal ? Oui, papa. Nina arrive près de la toile. Elle regarde les fraises, puis la poule. Une plume jaune tient sous la toile. La plume, papa. Tu la vois, la plume ? Oui, jaune. En ce moment, Raphaël veut dire le mot. Je le dis, maintenant ! Le mot de la poule, tout de suite. Tu le connais, Raphaël ? Oui, maman. J'ai vu. Nina s'arrête. Ses lèvres bougent, sans le mot. Raphaël connaît le mot. Il ouvre la bouche. Poule ! Nina baisse les yeux. Ses épaules se serrent. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nina, Raphaël ? Oui, papa. Ta bouche est ouverte, Raphaël ? Un peu, maman. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le bord, un instant. L'éclat d'étal tremble, puis tient. L'éclat, papa ? Tu le vois, toi ? Oui, sur le bord.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Les tentes du marché claquent un peu au vent. Une caisse de fraises est rouge comme des perles. Un sac en papier froisse, crac. Au loin, une poule fait cot-cot. Ça sent la terre et le pain. On reste près de moi, Mila. Tu tiens le bord du panier ? Oui, papa. Il est rêche. En ce moment, Mila marche entre les étals. Le sol est un peu collant, entre les caisses. On s'arrête près des fraises. Elles sentent fort, tu trouves ? Oui. Elles sont toutes rouges. Aniss marche à côté, le sac à la main. Une plume jaune a glissé sous une caisse. J'ai vu... Aniss s'arrête. Il cherche le mot. Mila a entendu la poule, elle aussi. Elle ouvre la bouche. On peut laisser le temps, Mila. On attend la fin de la phrase. Mila referme la bouche. Elle tient le panier plus fort. Elle compte dans sa tête. Un. Deux. Trois. Le sac d'Aniss froisse encore. J'ai vu une poule. Elle faisait cot-cot. Oui. Cot-cot. Bravo, Mila. Tu as su attendre. Ils avancent vers les poires. Les poires sont vertes, un peu bosselées. Je veux... Aniss cherche encore. Mila attend encore. Une tente claque au-dessus d'eux. Je veux une poire. Une poire, d'accord. Mila, tu as écouté jusqu'au bout ? Oui, papa. On laisse le temps. Papa prend une poire dans le papier. Le papier est un peu rêche aussi. Elle est... Mila attend la fin. Elle est douce. Douce, oui. Vous parlez l'un après l'autre. On a fini près de cet étal ? Oui. On peut rentrer. Le panier est un peu lourd, maintenant. Les fraises sentent fort, tout près. On compte les poires, Mila ? Une. Deux. Et... Mila attend. Et trois. Tu as encore attendu la fin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte glisse sur le métal de la balance. Elle brille, papa. Tu la vois, Raphaël ? Oui, papa. La goutte s'étire, puis tombe sur la toile. Elle a fait un rond. La toile est tendue, Raphaël ? Oui, maman. Ça sent le pain chaud, tout près. Ça sent le pain, papa. Tu le sens, toi ? Oui, fort. Des fraises rouges tiennent sur la toile. Elles sont lisses. Elles sentent fort, tu trouves ? Oui, maman. Au bord, un &lt;emphasis level="moderate"&gt;éclat d'étal&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, ce petit point ? Oui, un petit point. Un sac en papier froisse, crac. Il est rêche. Tu le tiens, Raphaël ? Oui, maman. Au loin, une poule fait cot-cot. J'entends la poule ! Elle est derrière l'étal ? Oui, papa. Nina arrive près de la toile. Elle regarde les fraises, puis la poule. Une plume jaune tient sous la toile. La plume, papa. Tu la vois, la plume ? Oui, jaune. En ce moment, Raphaël veut dire le mot. Je le dis, maintenant ! Le mot de la poule, tout de suite. Tu le connais, Raphaël ? Oui, maman. J'ai vu. Nina s'arrête. Ses lèvres bougent, sans le mot. Raphaël connaît le mot. Il ouvre la bouche. Poule ! Nina baisse les yeux. Ses épaules se serrent. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nina, Raphaël ? Oui, papa. Ta bouche est ouverte, Raphaël ? Un peu, maman. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le bord, un instant. L'éclat d'étal tremble, puis tient. L'éclat, papa ? Tu le vois, toi ? Oui, sur le bord.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Octave est au marché avec papa. Tess veut raconter. Elle dit : j'ai vu.. Puis elle cherche le mot. Octave connaît le mot. Il ouvre la bouche. Papa dit : on peut &lt;emphasis&gt;laisser&lt;/emphasis&gt; le temps. On n'achève pas à sa place. Octave attend la fin de la phrase. Tess respire. Elle dit : j'ai vu un canard. Octave sourit. Il a su laisser le temps. [pause]</t>
+          <t>Une goutte glisse sur le métal de la balance. Elle brille, papa. Tu la vois, Raphaël ? Oui, papa. La goutte s'étire, puis tombe sur la toile. Elle a fait un rond. La toile est tendue, Raphaël ? Oui, maman. Ça sent le pain chaud, tout près. Ça sent le pain, papa. Tu le sens, toi ? Oui, fort. Des fraises rouges tiennent sur la toile. Elles sont lisses. Elles sentent fort, tu trouves ? Oui, maman. Au bord, un &lt;emphasis&gt;éclat d'étal&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, ce petit point ? Oui, un petit point. Un sac en papier froisse, crac. Il est rêche. Tu le tiens, Raphaël ? Oui, maman. Au loin, une poule fait cot-cot. J'entends la poule ! Elle est derrière l'étal ? Oui, papa. Nina arrive près de la toile. Elle regarde les fraises, puis la poule. Une plume jaune tient sous la toile. La plume, papa. Tu la vois, la plume ? Oui, jaune. En ce moment, Raphaël veut dire le mot. Je le dis, maintenant ! Le mot de la poule, tout de suite. Tu le connais, Raphaël ? Oui, maman. J'ai vu. Nina s'arrête. Ses lèvres bougent, sans le mot. Raphaël connaît le mot. Il ouvre la bouche. Poule ! Nina baisse les yeux. Ses épaules se serrent. Oh. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nina, Raphaël ? Oui, papa. Ta bouche est ouverte, Raphaël ? Un peu, maman. Raphaël refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le bord, un instant. L'éclat d'étal tremble, puis tient. L'éclat, papa ? Tu le vois, toi ? Oui, sur le bord. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>laisser</t>
+          <t>éclat d'étal</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,76 +1321,82 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_connait_le_mot_ouvre_la_bouche; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les tentes du marché claquent un peu au vent.
-narrateur|Une caisse de fraises est rouge comme des perles.
+          <t>narrateur|Une goutte glisse sur le métal de la balance.
+enfant-m|Elle brille, papa.
+papa|Tu la vois, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|La goutte s'étire, puis tombe sur la toile.
+enfant-m|Elle a fait un rond.
+maman|La toile est tendue, Raphaël ?
+enfant-m|Oui, maman.
+narrateur|Ça sent le pain chaud, tout près.
+enfant-m|Ça sent le pain, papa.
+papa|Tu le sens, toi ?
+enfant-m|Oui, fort.
+narrateur|Des fraises rouges tiennent sur la toile.
+enfant-m|Elles sont lisses.
+maman|Elles sentent fort, tu trouves ?
+enfant-m|Oui, maman.
+narrateur|Au bord, un éclat d'étal brille.
+enfant-m|Il brille, papa.
+papa|Tu le vois, ce petit point ?
+enfant-m|Oui, un petit point.
 narrateur|Un sac en papier froisse, crac.
+enfant-m|Il est rêche.
+maman|Tu le tiens, Raphaël ?
+enfant-m|Oui, maman.
 narrateur|Au loin, une poule fait cot-cot.
-narrateur|Ça sent la terre et le pain.
-papa|On reste près de moi, Mila.
-papa|Tu tiens le bord du panier ?
-enfant-f|Oui, papa.
-enfant-f|Il est rêche.
-narrateur|En ce moment, Mila marche entre les étals.
-narrateur|Le sol est un peu collant, entre les caisses.
-papa|On s'arrête près des fraises.
-papa|Elles sentent fort, tu trouves ?
-enfant-f|Oui.
-enfant-f|Elles sont toutes rouges.
-narrateur|Aniss marche à côté, le sac à la main.
-narrateur|Une plume jaune a glissé sous une caisse.
-copain|J'ai vu...
-narrateur|Aniss s'arrête.
-narrateur|Il cherche le mot.
-narrateur|Mila a entendu la poule, elle aussi.
-narrateur|Elle ouvre la bouche.
-papa|On peut laisser le temps, Mila.
-papa|On attend la fin de la phrase.
-narrateur|Mila referme la bouche.
-narrateur|Elle tient le panier plus fort.
-narrateur|Elle compte dans sa tête.
-narrateur|Un.
-narrateur|Deux.
-narrateur|Trois.
-narrateur|Le sac d'Aniss froisse encore.
-copain|J'ai vu une poule.
-enfant-f|Elle faisait cot-cot.
-copain|Oui.
-copain|Cot-cot.
-papa|Bravo, Mila.
-papa|Tu as su attendre.
-narrateur|Ils avancent vers les poires.
-narrateur|Les poires sont vertes, un peu bosselées.
-copain|Je veux...
-narrateur|Aniss cherche encore.
-narrateur|Mila attend encore.
-narrateur|Une tente claque au-dessus d'eux.
-copain|Je veux une poire.
-papa|Une poire, d'accord.
-papa|Mila, tu as écouté jusqu'au bout ?
-enfant-f|Oui, papa.
-papa|On laisse le temps.
-narrateur|Papa prend une poire dans le papier.
-narrateur|Le papier est un peu rêche aussi.
-copain|Elle est...
-narrateur|Mila attend la fin.
-copain|Elle est douce.
-enfant-f|Douce, oui.
-papa|Vous parlez l'un après l'autre.
-papa|On a fini près de cet étal ?
-enfant-f|Oui.
-enfant-f|On peut rentrer.
-narrateur|Le panier est un peu lourd, maintenant.
-narrateur|Les fraises sentent fort, tout près.
-papa|On compte les poires, Mila ?
-enfant-f|Une.
-enfant-f|Deux.
-copain|Et...
-narrateur|Mila attend.
-copain|Et trois.
-papa|Tu as encore attendu la fin.</t>
+enfant-m|J'entends la poule !
+papa|Elle est derrière l'étal ?
+enfant-m|Oui, papa.
+narrateur|Nina arrive près de la toile.
+narrateur|Elle regarde les fraises, puis la poule.
+narrateur|Une plume jaune tient sous la toile.
+enfant-m|La plume, papa.
+papa|Tu la vois, la plume ?
+enfant-m|Oui, jaune.
+narrateur|En ce moment, Raphaël veut dire le mot.
+enfant-m|Je le dis, maintenant !
+enfant-m|Le mot de la poule, tout de suite.
+maman|Tu le connais, Raphaël ?
+enfant-m|Oui, maman.
+copine|J'ai vu.
+narrateur|Nina s'arrête.
+narrateur|Ses lèvres bougent, sans le mot.
+narrateur|Raphaël connaît le mot.
+narrateur|Il ouvre la bouche.
+enfant-m|Poule !
+narrateur|Nina baisse les yeux.
+narrateur|Ses épaules se serrent.
+enfant-m|Oh.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Nina, Raphaël ?
+enfant-m|Oui, papa.
+maman|Ta bouche est ouverte, Raphaël ?
+enfant-m|Un peu, maman.
+narrateur|Raphaël refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe le bord, un instant.
+narrateur|L'éclat d'étal tremble, puis tient.
+enfant-m|L'éclat, papa ?
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le bord.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>balance,toile</t>
         </is>
       </c>
     </row>
@@ -1417,17 +1423,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Aniss cherche un mot. Que fait Mila ?</t>
+          <t>Nina cherche un mot. Que fait Raphaël ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aniss cherche un mot. Que fait Mila ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Nina&lt;/emphasis&gt; cherche un mot. Que fait Raphaël ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Tess cherche un mot. Que fait Octave ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Nina&lt;/emphasis&gt; cherche un mot. Que fait Raphaël ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1490,18 +1496,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1516,34 +1522,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Nina</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1552,29 +1562,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=nina_cherche_un_mot_que_fait_raphael; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Aniss cherche un mot.
-narrateur|Que fait Mila ?</t>
+          <t>narrateur|Nina cherche un mot.
+narrateur|Que fait Raphaël ?</t>
         </is>
       </c>
     </row>
@@ -1601,17 +1611,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila a su laisser le temps. Aniss a fini sa phrase. On attend la fin de la phrase. Bravo, Mila. J'ai laissé le temps.</t>
+          <t>Raphaël tient le sac, sans parler. Sa bouche reste fermée. Il attend. Nina respire, un peu plus large. J'ai vu une poule. Une poule. Elle faisait cot-cot. Cot-cot. Tu l'as entendue, Raphaël ? Oui, papa. Tu as entendu Nina ? Oui, maman. Le ventre de Raphaël se desserre. Merci, Raphaël. Maman a vu la bouche fermée. Les poires sont plus loin ? Oui, papa. Ils avancent vers les poires. Les poires sont vertes, un peu bosselées. Elles sont dures. Tu les touches, Raphaël ? Un peu, maman. Un éclat d'étal luit au bord. Le point, papa. Sur la toile, Raphaël ? Oui, il tient. Le sac froisse contre la jambe. Il est rêche, maman. On le garde ouvert ? Oui, maman. Le sol colle un peu, sous les pas. Il colle, papa. Tu le sens, le sol ? Oui. Nina marche à côté, le sac trop grand. Elle tient le bord. Le papier est tiède, à cause du soleil. Il est chaud, maman. Le soleil est dessus ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila a su laisser le temps. Aniss a fini sa phrase. On attend la fin de la phrase. Bravo, Mila. J'ai laissé le temps.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël tient le sac, sans parler. Sa bouche reste fermée. Il &lt;emphasis level="moderate"&gt;attend&lt;/emphasis&gt;. Nina respire, un peu plus large. J'ai vu une poule. Une poule. Elle faisait cot-cot. Cot-cot. Tu l'as entendue, Raphaël ? Oui, papa. Tu as entendu Nina ? Oui, maman. Le ventre de Raphaël se desserre. Merci, Raphaël. Maman a vu la bouche fermée. Les poires sont plus loin ? Oui, papa. Ils avancent vers les poires. Les poires sont vertes, un peu bosselées. Elles sont dures. Tu les touches, Raphaël ? Un peu, maman. Un éclat d'étal luit au bord. Le point, papa. Sur la toile, Raphaël ? Oui, il tient. Le sac froisse contre la jambe. Il est rêche, maman. On le garde ouvert ? Oui, maman. Le sol colle un peu, sous les pas. Il colle, papa. Tu le sens, le sol ? Oui. Nina marche à côté, le sac trop grand. Elle tient le bord. Le papier est tiède, à cause du soleil. Il est chaud, maman. Le soleil est dessus ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Octave a su &lt;emphasis&gt;laisser&lt;/emphasis&gt; le temps. Tess a fini sa phrase. [pause]</t>
+          <t>Raphaël tient le sac, sans parler. Sa bouche reste fermée. Il &lt;emphasis&gt;attend&lt;/emphasis&gt;. Nina respire, un peu plus large. J'ai vu une poule. Une poule. Elle faisait cot-cot. Cot-cot. Tu l'as entendue, Raphaël ? Oui, papa. Tu as entendu Nina ? Oui, maman. Le ventre de Raphaël se desserre. Merci, Raphaël. Maman a vu la bouche fermée. Les poires sont plus loin ? Oui, papa. Ils avancent vers les poires. Les poires sont vertes, un peu bosselées. Elles sont dures. Tu les touches, Raphaël ? Un peu, maman. Un éclat d'étal luit au bord. Le point, papa. Sur la toile, Raphaël ? Oui, il tient. Le sac froisse contre la jambe. Il est rêche, maman. On le garde ouvert ? Oui, maman. Le sol colle un peu, sous les pas. Il colle, papa. Tu le sens, le sol ? Oui. Nina marche à côté, le sac trop grand. Elle tient le bord. Le papier est tiède, à cause du soleil. Il est chaud, maman. Le soleil est dessus ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1658,7 +1668,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1666,10 +1676,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1692,30 +1702,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>laisser</t>
+          <t>attend</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1724,10 +1734,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1740,16 +1750,56 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_referme_la_bouche_attend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Mila a su laisser le temps.
-narrateur|Aniss a fini sa phrase.
-papa|On attend la fin de la phrase.
-papa|Bravo, Mila.
-enfant-f|J'ai laissé le temps.</t>
+          <t>narrateur|Raphaël tient le sac, sans parler.
+narrateur|Sa bouche reste fermée.
+narrateur|Il attend.
+narrateur|Nina respire, un peu plus large.
+copine|J'ai vu une poule.
+enfant-m|Une poule.
+copine|Elle faisait cot-cot.
+enfant-m|Cot-cot.
+papa|Tu l'as entendue, Raphaël ?
+enfant-m|Oui, papa.
+maman|Tu as entendu Nina ?
+enfant-m|Oui, maman.
+narrateur|Le ventre de Raphaël se desserre.
+maman|Merci, Raphaël.
+narrateur|Maman a vu la bouche fermée.
+papa|Les poires sont plus loin ?
+enfant-m|Oui, papa.
+narrateur|Ils avancent vers les poires.
+narrateur|Les poires sont vertes, un peu bosselées.
+enfant-m|Elles sont dures.
+maman|Tu les touches, Raphaël ?
+enfant-m|Un peu, maman.
+narrateur|Un éclat d'étal luit au bord.
+enfant-m|Le point, papa.
+papa|Sur la toile, Raphaël ?
+enfant-m|Oui, il tient.
+narrateur|Le sac froisse contre la jambe.
+enfant-m|Il est rêche, maman.
+maman|On le garde ouvert ?
+enfant-m|Oui, maman.
+narrateur|Le sol colle un peu, sous les pas.
+enfant-m|Il colle, papa.
+papa|Tu le sens, le sol ?
+enfant-m|Oui.
+narrateur|Nina marche à côté, le sac trop grand.
+enfant-m|Elle tient le bord.
+narrateur|Le papier est tiède, à cause du soleil.
+enfant-m|Il est chaud, maman.
+maman|Le soleil est dessus ?
+enfant-m|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>sac,poule</t>
         </is>
       </c>
     </row>
@@ -1776,17 +1826,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Papa achète une poire. Tu donnes la main, Mila ? Oui, papa. Mila donne la main. Aniss porte le petit sac. On rentre. Doucement, entre les tentes. La poule, elle... Mila attend encore une fois. La poule, elle est restée. Oui. Au marché. Tu as encore laissé le temps. La poule fait encore cot-cot, au loin.</t>
+          <t>Ils s'arrêtent près des poires. Je prends, maintenant ! Raphaël avance le sac trop vite. Le papier froisse trop fort. Nina recule d'un pas. Oh. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe une poire, un instant. La toile claque, légère. Il revoit l'éclat d'étal. Une tente claque au-dessus d'eux. Je veux. Nina sursaute. Le mot tombe. Raphaël connaît le mot. Il ouvre la bouche. Puis il la referme. Il attend. Je veux une poire. Une poire, Raphaël ? Oui, papa. Papa prend une poire dans le papier. Le papier est rêche, contre les doigts. Elle est. Nina s'arrête. Raphaël garde la bouche fermée. Elle est douce. Douce, oui. Tes mains tiennent le sac, Raphaël ? Oui, maman. On a la poire, vous deux ? Oui, papa. Nina souffle, longuement. Elle a dit, papa. Tu l'as vue, toi ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Papa achète une poire. Tu donnes la main, Mila ? Oui, papa. Mila donne la main. Aniss porte le petit sac. On rentre. Doucement, entre les tentes. La poule, elle... Mila attend encore une fois. La poule, elle est restée. Oui. Au marché. Tu as encore laissé le temps. La poule fait encore cot-cot, au loin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils s'arrêtent près des poires. Je prends, maintenant ! Raphaël avance le sac trop vite. Le papier froisse trop fort. Nina recule d'un pas. Oh. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe une poire, un instant. La toile claque, légère. Il revoit l'&lt;emphasis level="moderate"&gt;éclat d'étal&lt;/emphasis&gt;. Une tente claque au-dessus d'eux. Je veux. Nina sursaute. Le mot tombe. Raphaël connaît le mot. Il ouvre la bouche. Puis il la referme. Il attend. Je veux une poire. Une poire, Raphaël ? Oui, papa. Papa prend une poire dans le papier. Le papier est rêche, contre les doigts. Elle est. Nina s'arrête. Raphaël garde la bouche fermée. Elle est douce. Douce, oui. Tes mains tiennent le sac, Raphaël ? Oui, maman. On a la poire, vous deux ? Oui, papa. Nina souffle, longuement. Elle a dit, papa. Tu l'as vue, toi ? Oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Papa achète une poire. Octave donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Ils s'arrêtent près des poires. Je prends, maintenant ! Raphaël avance le sac trop vite. Le papier froisse trop fort. Nina recule d'un pas. Oh. Raphaël refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe une poire, un instant. La toile claque, légère. Il revoit l'&lt;emphasis&gt;éclat d'étal&lt;/emphasis&gt;. Une tente claque au-dessus d'eux. Je veux. Nina sursaute. Le mot tombe. Raphaël connaît le mot. Il ouvre la bouche. Puis il la referme. Il attend. Je veux une poire. Une poire, Raphaël ? Oui, papa. Papa prend une poire dans le papier. Le papier est rêche, contre les doigts. Elle est. Nina s'arrête. Raphaël garde la bouche fermée. Elle est douce. Douce, oui. Tes mains tiennent le sac, Raphaël ? Oui, maman. On a la poire, vous deux ? Oui, papa. Nina souffle, longuement. Elle a dit, papa. Tu l'as vue, toi ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1833,7 +1883,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1841,10 +1891,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1867,30 +1917,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat d'étal</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1899,10 +1949,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1913,23 +1963,56 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=sac_trop_vite_mot_qui_tombe_il_referme; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Papa achète une poire.
-papa|Tu donnes la main, Mila ?
-enfant-f|Oui, papa.
-narrateur|Mila donne la main.
-narrateur|Aniss porte le petit sac.
-papa|On rentre.
-papa|Doucement, entre les tentes.
-copain|La poule, elle...
-narrateur|Mila attend encore une fois.
-copain|La poule, elle est restée.
-enfant-f|Oui.
-enfant-f|Au marché.
-papa|Tu as encore laissé le temps.
-narrateur|La poule fait encore cot-cot, au loin.</t>
+          <t>narrateur|Ils s'arrêtent près des poires.
+enfant-m|Je prends, maintenant !
+narrateur|Raphaël avance le sac trop vite.
+narrateur|Le papier froisse trop fort.
+narrateur|Nina recule d'un pas.
+enfant-m|Oh.
+narrateur|Raphaël refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe une poire, un instant.
+narrateur|La toile claque, légère.
+narrateur|Il revoit l'éclat d'étal.
+narrateur|Une tente claque au-dessus d'eux.
+copine|Je veux.
+narrateur|Nina sursaute.
+narrateur|Le mot tombe.
+narrateur|Raphaël connaît le mot.
+narrateur|Il ouvre la bouche.
+narrateur|Puis il la referme.
+narrateur|Il attend.
+copine|Je veux une poire.
+papa|Une poire, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Papa prend une poire dans le papier.
+narrateur|Le papier est rêche, contre les doigts.
+copine|Elle est.
+narrateur|Nina s'arrête.
+narrateur|Raphaël garde la bouche fermée.
+copine|Elle est douce.
+enfant-m|Douce, oui.
+maman|Tes mains tiennent le sac, Raphaël ?
+enfant-m|Oui, maman.
+papa|On a la poire, vous deux ?
+enfant-m|Oui, papa.
+narrateur|Nina souffle, longuement.
+enfant-m|Elle a dit, papa.
+papa|Tu l'as vue, toi ?
+enfant-m|Oui.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>tente,sac</t>
         </is>
       </c>
     </row>
@@ -1956,17 +2039,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo. La poire roule un peu dans le panier.</t>
+          <t>Ils restent près de la toile. La poule est restée, Raphaël ? Oui, maman. Tu donnes la main, Raphaël ? Oui, papa. Raphaël donne la main. Nina porte le petit sac. La poire est dedans. Poule. Poule. Le sac est un peu lourd ? Un peu, papa. On rentre entre les tentes ? Oui, maman. Au loin, la poule fait cot-cot. Je l'entends. Un éclat d'étal tient au bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai attendu la fin. Bravo. La poire roule un peu dans le panier.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la toile. La poule est restée, Raphaël ? Oui, maman. Tu donnes la main, Raphaël ? Oui, papa. Raphaël donne la main. Nina porte le petit sac. La poire est dedans. Poule. Poule. Le sac est un peu lourd ? Un peu, papa. On rentre entre les tentes ? Oui, maman. Au loin, la poule fait cot-cot. Je l'entends. Un &lt;emphasis level="moderate"&gt;éclat d'étal&lt;/emphasis&gt; tient au bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la toile. La poule est restée, Raphaël ? Oui, maman. Tu donnes la main, Raphaël ? Oui, papa. Raphaël donne la main. Nina porte le petit sac. La poire est dedans. Poule. Poule. Le sac est un peu lourd ? Un peu, papa. On rentre entre les tentes ? Oui, maman. Au loin, la poule fait cot-cot. Je l'entends. Un &lt;emphasis&gt;éclat d'étal&lt;/emphasis&gt; tient au bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2013,18 +2096,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2033,12 +2116,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2047,17 +2130,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'étal</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2066,11 +2153,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2079,26 +2166,49 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_au_bord; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai attendu la fin.
-papa|Bravo.
-narrateur|La poire roule un peu dans le panier.</t>
+          <t>narrateur|Ils restent près de la toile.
+maman|La poule est restée, Raphaël ?
+enfant-m|Oui, maman.
+papa|Tu donnes la main, Raphaël ?
+enfant-m|Oui, papa.
+narrateur|Raphaël donne la main.
+narrateur|Nina porte le petit sac.
+enfant-m|La poire est dedans.
+copine|Poule.
+enfant-m|Poule.
+papa|Le sac est un peu lourd ?
+enfant-m|Un peu, papa.
+maman|On rentre entre les tentes ?
+enfant-m|Oui, maman.
+narrateur|Au loin, la poule fait cot-cot.
+enfant-m|Je l'entends.
+narrateur|Un éclat d'étal tient au bord.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>toile</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2183,6 +2293,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>